<commit_message>
Polish examples with unique names and three-digit extensions
</commit_message>
<xml_diff>
--- a/assets/ssemsearch-template.xlsx
+++ b/assets/ssemsearch-template.xlsx
@@ -25422,9 +25422,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A7"/>
-  <cols>
-    <col min="1" max="1" width="100.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -25438,7 +25435,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>내선 열 C2:C5001은 텍스트 형식입니다. 0231처럼 앞자리 0을 포함해 입력하세요.</v>
+        <v>내선 열 C2:C5001은 텍스트 형식입니다. 031처럼 앞자리 0을 포함해 입력하세요.</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Release v1.1.0 with AI import guidance and updated downloads
</commit_message>
<xml_diff>
--- a/assets/ssemsearch-template.xlsx
+++ b/assets/ssemsearch-template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="교직원 명단" sheetId="1" r:id="rId1"/>
+    <sheet name="명단" sheetId="1" r:id="rId1"/>
     <sheet name="작성안내" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
@@ -400,19 +400,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C5001"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>이름</v>
       </c>
       <c r="B1" t="str">
-        <v>교무실</v>
+        <v>위치(부서)</v>
       </c>
       <c r="C1" t="str">
         <v>내선번호</v>
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
       <c r="C2" s="1" t="str">
         <v/>
       </c>
@@ -25422,6 +25433,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A7"/>
+  <cols>
+    <col min="1" max="1" width="90.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -25430,32 +25444,32 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>교직원 명단 시트의 2행부터 이름, 교무실, 내선번호를 입력하세요.</v>
+        <v>명단 시트의 2행부터 이름, 위치(부서), 내선번호를 입력하세요. 빈 셀이 있어도 나머지 정보로 등록할 수 있습니다.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>내선 열 C2:C5001은 텍스트 형식입니다. 031처럼 앞자리 0을 포함해 입력하세요.</v>
+        <v>내선번호는 숫자 문자 1~20자리입니다. 이 양식의 C2:C5001은 텍스트 형식으로 준비되어 있습니다.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>기존 숫자 셀에서 이미 사라진 앞자리 0은 자동으로 복원되지 않습니다.</v>
+        <v>기존 파일을 사용한다면 내선 열 전체를 텍스트 형식으로 지정하세요.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>병합 셀, 수식, 날짜, 오류 셀과 필수값 누락을 수정해 주세요.</v>
+        <v>앞자리 0을 보존하려면 0231처럼 텍스트로 입력하세요.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>.xlsx, 10MB 이하, 머리글 아래 데이터 영역 5000행 및 100열 이하를 지원합니다.</v>
+        <v>병합 셀, 수식, 날짜, 오류 셀은 사용할 수 없습니다.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>새 명단을 가져오면 기존 명단 전체를 교체합니다.</v>
+        <v>최대 5,000명, 100열, 10MB의 .xlsx 파일을 지원합니다.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>